<commit_message>
Added o4-mini Fine-Tuned Results for Python
</commit_message>
<xml_diff>
--- a/CWEsIntroducedMapping/CWEMappings.xlsx
+++ b/CWEsIntroducedMapping/CWEMappings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EducationalFiles\Massey\MInfSc\Re\Scenarios\CWEsIntroducedMapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5459FD-C915-4C39-87F0-997047FFAA73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3363576C-CD53-45B2-8969-82D0E3263752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13866" xr2:uid="{E9D892D6-17AD-44AD-B269-50B4899FCA39}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="34">
   <si>
     <t>GPT 4.1</t>
   </si>
@@ -132,9 +132,6 @@
   </si>
   <si>
     <t>[502], [79, 116]</t>
-  </si>
-  <si>
-    <t>xx</t>
   </si>
   <si>
     <t>Python</t>
@@ -527,7 +524,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.5">
@@ -554,7 +551,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.5">
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -783,7 +780,7 @@
         <v>17</v>
       </c>
       <c r="E28" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.5">
@@ -797,7 +794,7 @@
         <v>9</v>
       </c>
       <c r="E29" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.5">
@@ -811,7 +808,7 @@
         <v>17</v>
       </c>
       <c r="E30" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>